<commit_message>
Polish employer job posting experience
</commit_message>
<xml_diff>
--- a/documentation/CareerConnect_Project_Planning_Master_Report.xlsx
+++ b/documentation/CareerConnect_Project_Planning_Master_Report.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\liqae\job-portal-main\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6639B7A0-61A4-4474-9695-EB2D0F2EBCD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{695EFDB4-E439-4352-AD75-F6371596D3E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10875" yWindow="3885" windowWidth="12300" windowHeight="9360" firstSheet="3" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Executive_Summary" sheetId="1" r:id="rId1"/>
@@ -1528,14 +1528,14 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1853,50 +1853,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="39.950000000000003" customHeight="1">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
     </row>
     <row r="3" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A3" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="11"/>
+      <c r="B3" s="13"/>
       <c r="C3" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="11"/>
+      <c r="D3" s="13"/>
       <c r="E3" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="11"/>
+      <c r="F3" s="13"/>
       <c r="G3" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="H3" s="11"/>
+      <c r="H3" s="13"/>
     </row>
     <row r="4" spans="1:8" ht="27.95" customHeight="1">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="11"/>
-      <c r="C4" s="10" t="s">
+      <c r="B4" s="13"/>
+      <c r="C4" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="11"/>
-      <c r="E4" s="10" t="s">
+      <c r="D4" s="13"/>
+      <c r="E4" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="F4" s="11"/>
-      <c r="G4" s="10" t="s">
+      <c r="F4" s="13"/>
+      <c r="G4" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="11"/>
+      <c r="H4" s="13"/>
     </row>
     <row r="6" spans="1:8" ht="18.75">
       <c r="A6" s="1" t="s">
@@ -2046,15 +2046,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="39.950000000000003" customHeight="1">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
     </row>
     <row r="3" spans="1:7" ht="27.95" customHeight="1">
       <c r="A3" s="2" t="s">
@@ -2277,13 +2277,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="39.950000000000003" customHeight="1">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
     </row>
     <row r="3" spans="1:5" ht="27.95" customHeight="1">
       <c r="A3" s="2" t="s">
@@ -2409,14 +2409,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="39.950000000000003" customHeight="1">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
     </row>
     <row r="3" spans="1:6" ht="27.95" customHeight="1">
       <c r="A3" s="2" t="s">
@@ -2783,17 +2783,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="39.950000000000003" customHeight="1">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="10" t="s">
         <v>149</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="11"/>
+      <c r="I1" s="11"/>
     </row>
     <row r="3" spans="1:9" ht="27.95" customHeight="1">
       <c r="A3" s="2" t="s">
@@ -3863,16 +3863,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="39.950000000000003" customHeight="1">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="10" t="s">
         <v>282</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="11"/>
     </row>
     <row r="3" spans="1:8" ht="27.95" customHeight="1">
       <c r="A3" s="2" t="s">
@@ -3900,7 +3900,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="26.1" customHeight="1">
+    <row r="4" spans="1:8" ht="30">
       <c r="A4" s="9">
         <v>1</v>
       </c>
@@ -3952,7 +3952,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="26.1" customHeight="1">
+    <row r="6" spans="1:8" ht="30">
       <c r="A6" s="9">
         <v>3</v>
       </c>
@@ -3978,7 +3978,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="26.1" customHeight="1">
+    <row r="7" spans="1:8" ht="30">
       <c r="A7" s="9">
         <v>4</v>
       </c>
@@ -4004,7 +4004,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="26.1" customHeight="1">
+    <row r="8" spans="1:8" ht="30">
       <c r="A8" s="9">
         <v>5</v>
       </c>
@@ -4030,7 +4030,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="26.1" customHeight="1">
+    <row r="9" spans="1:8" ht="30">
       <c r="A9" s="9">
         <v>6</v>
       </c>
@@ -4056,7 +4056,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="26.1" customHeight="1">
+    <row r="10" spans="1:8" ht="30">
       <c r="A10" s="9">
         <v>7</v>
       </c>
@@ -4082,7 +4082,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="26.1" customHeight="1">
+    <row r="11" spans="1:8" ht="30">
       <c r="A11" s="9">
         <v>8</v>
       </c>
@@ -4108,7 +4108,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="26.1" customHeight="1">
+    <row r="12" spans="1:8" ht="30">
       <c r="A12" s="9">
         <v>9</v>
       </c>
@@ -4157,17 +4157,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="39.950000000000003" customHeight="1">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="10" t="s">
         <v>332</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="11"/>
+      <c r="I1" s="11"/>
     </row>
     <row r="3" spans="1:9" ht="27.95" customHeight="1">
       <c r="A3" s="2" t="s">

</xml_diff>